<commit_message>
Updates to contrail avoidance calculation
</commit_message>
<xml_diff>
--- a/data/250428_Abatement costs synfuels blue hydrogen.xlsx
+++ b/data/250428_Abatement costs synfuels blue hydrogen.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/ydubey_ethz_ch/Documents/Documents/GitHub/DACCSvDACCU/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="436" documentId="8_{00D5806A-E842-4966-A868-24FDBCA4DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CB971F3-BD3A-40AA-895B-C074B0FE06A3}"/>
+  <xr:revisionPtr revIDLastSave="437" documentId="8_{00D5806A-E842-4966-A868-24FDBCA4DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B09F501-8615-4277-ABA4-BD431A1F6A41}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9A4A7CCA-7739-4C0E-9453-6B3361FAEDB6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{9A4A7CCA-7739-4C0E-9453-6B3361FAEDB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="2" r:id="rId1"/>
@@ -40,6 +40,24 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={B30D06FA-549B-4880-9132-62D731C4599B}</author>
+  </authors>
+  <commentList>
+    <comment ref="C33" authorId="0" shapeId="0" xr:uid="{B30D06FA-549B-4880-9132-62D731C4599B}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This is varied between the 25% and 75% input cost as mentioned in red. For green hydrogen, the code automatically reads from 25% and 75% input cost. </t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="104">
   <si>
@@ -362,7 +380,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -475,6 +493,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -817,6 +841,12 @@
 </externalLink>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Dubey  Yash" id="{BF3000E7-5871-4931-863E-623DE601BC2A}" userId="S::ydubey@ethz.ch::8ec4c660-c9fe-4bb6-9560-48a212ff7621" providerId="AD"/>
+</personList>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1132,8 +1162,16 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C33" dT="2025-05-13T14:55:34.64" personId="{BF3000E7-5871-4931-863E-623DE601BC2A}" id="{B30D06FA-549B-4880-9132-62D731C4599B}">
+    <text xml:space="preserve">This is varied between the 25% and 75% input cost as mentioned in red. For green hydrogen, the code automatically reads from 25% and 75% input cost. </text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB317DF6-AD4E-4C2D-91E2-8E810E428F70}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB317DF6-AD4E-4C2D-91E2-8E810E428F70}">
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1684,6 +1722,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
changes for blue hydrogen based synfuels
Updated blue hydrogen based abatement cost
</commit_message>
<xml_diff>
--- a/data/250428_Abatement costs synfuels blue hydrogen.xlsx
+++ b/data/250428_Abatement costs synfuels blue hydrogen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/ydubey_ethz_ch/Documents/Documents/GitHub/DACCSvDACCU/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/ksievert_ethz_ch/Documents/SAF/_DACCS vs Synfuels/Python Code/DACCSvDACCU2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="437" documentId="8_{00D5806A-E842-4966-A868-24FDBCA4DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B09F501-8615-4277-ABA4-BD431A1F6A41}"/>
+  <xr:revisionPtr revIDLastSave="459" documentId="8_{00D5806A-E842-4966-A868-24FDBCA4DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A359AE4C-A908-4BA1-A590-DCC8B8A27938}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{9A4A7CCA-7739-4C0E-9453-6B3361FAEDB6}"/>
+    <workbookView xWindow="30" yWindow="-18120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{9A4A7CCA-7739-4C0E-9453-6B3361FAEDB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="2" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="108">
   <si>
     <t>Parameter</t>
   </si>
@@ -371,6 +371,18 @@
   </si>
   <si>
     <t>Median</t>
+  </si>
+  <si>
+    <t>50%</t>
+  </si>
+  <si>
+    <t>25%</t>
+  </si>
+  <si>
+    <t>75%</t>
+  </si>
+  <si>
+    <t>DACCS LCOR</t>
   </si>
 </sst>
 </file>
@@ -380,7 +392,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,12 +506,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -572,7 +578,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
@@ -644,6 +650,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1172,16 +1181,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB317DF6-AD4E-4C2D-91E2-8E810E428F70}">
-  <dimension ref="A1:K44"/>
-  <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K48"/>
+  <sheetFormatPr defaultColWidth="12.33203125" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" style="2"/>
+    <col min="1" max="1" width="17.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" style="2"/>
     <col min="3" max="3" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="12.28515625" style="2"/>
+    <col min="4" max="16384" width="12.33203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1195,7 +1204,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -1203,7 +1212,7 @@
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1212,7 +1221,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1221,7 +1230,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -1230,7 +1239,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1239,7 +1248,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -1247,7 +1256,7 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
@@ -1262,7 +1271,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
@@ -1277,7 +1286,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
@@ -1285,7 +1294,7 @@
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
@@ -1300,7 +1309,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>13</v>
       </c>
@@ -1315,7 +1324,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
@@ -1327,7 +1336,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
@@ -1339,7 +1348,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>18</v>
       </c>
@@ -1351,7 +1360,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1366,7 +1375,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>22</v>
       </c>
@@ -1374,7 +1383,7 @@
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>20</v>
       </c>
@@ -1389,7 +1398,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>23</v>
       </c>
@@ -1397,7 +1406,7 @@
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -1412,7 +1421,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -1427,7 +1436,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>24</v>
       </c>
@@ -1435,7 +1444,7 @@
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -1450,7 +1459,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -1465,7 +1474,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>25</v>
       </c>
@@ -1473,7 +1482,7 @@
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -1488,7 +1497,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -1503,7 +1512,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>26</v>
       </c>
@@ -1511,7 +1520,7 @@
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
@@ -1526,7 +1535,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -1541,7 +1550,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>27</v>
       </c>
@@ -1549,7 +1558,7 @@
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>28</v>
       </c>
@@ -1564,7 +1573,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="48" t="s">
         <v>28</v>
       </c>
@@ -1572,7 +1581,8 @@
         <v>2050</v>
       </c>
       <c r="C33" s="49">
-        <v>542</v>
+        <f>C48-25</f>
+        <v>517.75</v>
       </c>
       <c r="D33" s="48" t="s">
         <v>29</v>
@@ -1587,12 +1597,12 @@
       <c r="J33" s="50"/>
       <c r="K33" s="50"/>
     </row>
-    <row r="34" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="30" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>85</v>
       </c>
@@ -1609,7 +1619,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>85</v>
       </c>
@@ -1626,12 +1636,12 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="30" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="38" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="42" t="s">
         <v>88</v>
       </c>
@@ -1648,7 +1658,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="42" t="s">
         <v>88</v>
       </c>
@@ -1665,7 +1675,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="21" t="s">
         <v>38</v>
       </c>
@@ -1673,7 +1683,7 @@
       <c r="C40" s="23"/>
       <c r="D40" s="22"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
@@ -1687,7 +1697,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -1701,7 +1711,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="21" t="s">
         <v>66</v>
       </c>
@@ -1709,7 +1719,7 @@
       <c r="C43" s="22"/>
       <c r="D43" s="22"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>67</v>
       </c>
@@ -1718,6 +1728,33 @@
       </c>
       <c r="D44" s="2" t="s">
         <v>68</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="55" t="s">
+        <v>104</v>
+      </c>
+      <c r="B47" s="55" t="s">
+        <v>105</v>
+      </c>
+      <c r="C47" s="55" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="54">
+        <v>311.69281114021061</v>
+      </c>
+      <c r="B48" s="54">
+        <v>159.66348201703261</v>
+      </c>
+      <c r="C48" s="54">
+        <v>542.75</v>
       </c>
     </row>
   </sheetData>
@@ -1729,21 +1766,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24B4FBF-589B-4E3C-A2F1-4BB885F501FC}">
   <dimension ref="A1:K32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="47.7109375" customWidth="1"/>
-    <col min="2" max="4" width="31.7109375" customWidth="1"/>
-    <col min="5" max="5" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" customWidth="1"/>
+    <col min="1" max="1" width="47.6640625" customWidth="1"/>
+    <col min="2" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="36" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="36" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="36" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
@@ -1760,7 +1797,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>46</v>
       </c>
@@ -1777,7 +1814,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>31</v>
       </c>
@@ -1796,7 +1833,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>32</v>
       </c>
@@ -1814,7 +1851,7 @@
       </c>
       <c r="F5" s="45"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>72</v>
       </c>
@@ -1831,7 +1868,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="37" t="s">
         <v>74</v>
       </c>
@@ -1846,7 +1883,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="37" t="s">
         <v>75</v>
       </c>
@@ -1863,7 +1900,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>34</v>
       </c>
@@ -1880,7 +1917,7 @@
       </c>
       <c r="E9" s="33"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>35</v>
       </c>
@@ -1899,7 +1936,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -1935,7 +1972,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>59</v>
       </c>
@@ -1971,12 +2008,12 @@
         <v>102</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="18" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>69</v>
       </c>
@@ -1992,7 +2029,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>70</v>
       </c>
@@ -2008,7 +2045,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
         <v>71</v>
       </c>
@@ -2024,24 +2061,24 @@
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="44" t="s">
         <v>91</v>
       </c>
       <c r="B20" s="24"/>
       <c r="C20" s="24"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
     </row>
-    <row r="22" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="18" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="38" t="s">
         <v>79</v>
       </c>
@@ -2057,7 +2094,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>81</v>
       </c>
@@ -2073,22 +2110,22 @@
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="17"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="17"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
     </row>
-    <row r="27" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="18" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>62</v>
       </c>
@@ -2104,23 +2141,23 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>63</v>
       </c>
       <c r="B29" s="12">
         <f>(Inputs!$C$33/1000)*B13</f>
-        <v>1.225632097976177</v>
+        <v>1.1707952375039956</v>
       </c>
       <c r="C29" s="12">
         <f>(Inputs!$C$33/1000)*C13</f>
-        <v>1.8970000000000002</v>
+        <v>1.8121250000000002</v>
       </c>
       <c r="D29" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:11" s="52" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" s="52" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="52" t="s">
         <v>64</v>
       </c>
@@ -2138,34 +2175,34 @@
         <v>102</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>83</v>
       </c>
       <c r="B31" s="12">
         <f>B24*((Inputs!$C$33+Inputs!$C$36+Inputs!$C$39)/1000)</f>
-        <v>0.19600817322240002</v>
+        <v>0.18762510761280002</v>
       </c>
       <c r="C31" s="12">
         <f>C24*((Inputs!$C$33+Inputs!$C$36+Inputs!$C$39)/1000)</f>
-        <v>0.64317640464000003</v>
+        <v>0.61566841908000003</v>
       </c>
       <c r="D31" t="s">
         <v>21</v>
       </c>
       <c r="E31" s="19"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="17" t="s">
         <v>89</v>
       </c>
       <c r="B32" s="20">
         <f>SUM(B28:B31)</f>
-        <v>2.3413881981074187</v>
+        <v>2.2781682720256375</v>
       </c>
       <c r="C32" s="20">
         <f>SUM(C28:C31)</f>
-        <v>5.3151764046400007</v>
+        <v>5.2027934190800007</v>
       </c>
       <c r="D32" s="17" t="s">
         <v>21</v>
@@ -2189,24 +2226,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15B90E37-756A-4C57-9113-106741692D73}">
   <dimension ref="B2:F17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="97.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="55">
+    <row r="2" spans="2:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B2" s="56">
         <v>2050</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
       <c r="F2" s="40"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
         <v>0</v>
       </c>
@@ -2223,7 +2260,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="14" t="s">
         <v>49</v>
       </c>
@@ -2232,15 +2269,15 @@
       </c>
       <c r="D4" s="16">
         <f>'Study Parameters'!B32</f>
-        <v>2.3413881981074187</v>
+        <v>2.2781682720256375</v>
       </c>
       <c r="E4" s="16">
         <f>'Study Parameters'!C32</f>
-        <v>5.3151764046400007</v>
+        <v>5.2027934190800007</v>
       </c>
       <c r="F4" s="15"/>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="14" t="s">
         <v>50</v>
       </c>
@@ -2257,7 +2294,7 @@
       </c>
       <c r="F5" s="15"/>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="14" t="s">
         <v>90</v>
       </c>
@@ -2272,7 +2309,7 @@
       </c>
       <c r="F6" s="15"/>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="14" t="s">
         <v>52</v>
       </c>
@@ -2289,7 +2326,7 @@
       </c>
       <c r="F7" s="15"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="14" t="s">
         <v>53</v>
       </c>
@@ -2306,7 +2343,7 @@
       </c>
       <c r="F8" s="15"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="14" t="s">
         <v>53</v>
       </c>
@@ -2323,7 +2360,7 @@
       </c>
       <c r="F9" s="15"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="14" t="s">
         <v>100</v>
       </c>
@@ -2332,28 +2369,28 @@
       </c>
       <c r="D10" s="43">
         <f>(D4-D5) / D9 * 10^6</f>
-        <v>500.9439287508041</v>
+        <v>480.39774954323769</v>
       </c>
       <c r="E10" s="43">
         <f>(E4-E5) / E9 * 10^6</f>
-        <v>1467.4111362215485</v>
+        <v>1430.8871934663775</v>
       </c>
       <c r="F10" s="43">
         <f>MEDIAN(D10:E10)</f>
-        <v>984.17753248617623</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+        <v>955.64247150480765</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="51" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="51" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E17" s="54"/>
     </row>
   </sheetData>
@@ -2361,5 +2398,6 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Blue Hydrogen Calculation in Code
</commit_message>
<xml_diff>
--- a/data/250428_Abatement costs synfuels blue hydrogen.xlsx
+++ b/data/250428_Abatement costs synfuels blue hydrogen.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/ksievert_ethz_ch/Documents/SAF/_DACCS vs Synfuels/Python Code/DACCSvDACCU2/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/ydubey_ethz_ch/Documents/Documents/GitHub/DACCSvDACCU/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="459" documentId="8_{00D5806A-E842-4966-A868-24FDBCA4DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A359AE4C-A908-4BA1-A590-DCC8B8A27938}"/>
+  <xr:revisionPtr revIDLastSave="443" documentId="8_{00D5806A-E842-4966-A868-24FDBCA4DBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F13F146-0B66-43F8-A1F9-34CC89998825}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="-18120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{9A4A7CCA-7739-4C0E-9453-6B3361FAEDB6}"/>
+    <workbookView xWindow="-96" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{9A4A7CCA-7739-4C0E-9453-6B3361FAEDB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <externalReferences>
     <externalReference r:id="rId4"/>
   </externalReferences>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -58,8 +58,28 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={61935355-D025-4334-8AB7-9AFE8C085A31}</author>
+  </authors>
+  <commentList>
+    <comment ref="B18" authorId="0" shapeId="0" xr:uid="{61935355-D025-4334-8AB7-9AFE8C085A31}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    @Sievert  Katrin are these emissions measured in GWP100 or GWP20? Since the multipliers are 34x and 86x, there could be quite a significant difference between these. See section 3.1 for an example: https://www.sciencedirect.com/science/article/pii/S0306261921014215?via%3Dihub#b0215
+Reply:
+    Hi Yash, I used a GWP100 multiplier (36) - I didn't use a GWP20 multiplier for methane tho, fair point!</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="104">
   <si>
     <t>Parameter</t>
   </si>
@@ -151,61 +171,199 @@
     <t>$/tCO2</t>
   </si>
   <si>
+    <t>TO BE UPDATED WITH 25 AND 75TH RANGE OF DAC INPUT COSTS? SAME AS FOR SYNFUELS</t>
+  </si>
+  <si>
+    <t>CO2 Transport</t>
+  </si>
+  <si>
+    <t>CO2 Transport Cost</t>
+  </si>
+  <si>
+    <t>Dummy value for now</t>
+  </si>
+  <si>
+    <t>CO2 Storage</t>
+  </si>
+  <si>
+    <t>CO2 Storage Cost</t>
+  </si>
+  <si>
+    <t>NATURAL GAS</t>
+  </si>
+  <si>
+    <t>NG Price</t>
+  </si>
+  <si>
+    <t>$/GJ</t>
+  </si>
+  <si>
+    <t>Hydrogen Energy Content (Lower Heating Value, LV)</t>
+  </si>
+  <si>
+    <t>1 kg H2 in LHV basis</t>
+  </si>
+  <si>
+    <t>MJ</t>
+  </si>
+  <si>
+    <t>Key Parameters: Blue H₂ (SMR/ATR + CCS) + DAC</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
     <t>Source</t>
   </si>
   <si>
+    <t>Hydrogen Cost (€2022/kg H₂)</t>
+  </si>
+  <si>
+    <t>€2022/kg H₂</t>
+  </si>
+  <si>
+    <t>Frieden et al. (2024); 2050 SMR+CCS; Fig 5</t>
+  </si>
+  <si>
     <t>Hydrogen Cost ($/kg H₂)</t>
   </si>
   <si>
+    <t>$2023/kg H₂</t>
+  </si>
+  <si>
+    <t>Frieden et al. (2024)</t>
+  </si>
+  <si>
     <t>Hydrogen Production Emissions (kg CO₂/kg H₂)</t>
   </si>
   <si>
+    <t>kg CO₂/kg H₂</t>
+  </si>
+  <si>
+    <t>Katebah et al. (2022); 2.7: maximum carbon capture from the SMR plant using Option 1 is around 70% of the total CO2 emissions</t>
+  </si>
+  <si>
+    <t>NG consumption Methane</t>
+  </si>
+  <si>
+    <t>kg CH4/kg H2</t>
+  </si>
+  <si>
     <t>Katebah et al. (2022)</t>
   </si>
   <si>
+    <t>Methane GWP-100 potential (1 kg CH₄ = 36 kg CO₂e)</t>
+  </si>
+  <si>
+    <t>https://www.epa.gov/ghgemissions/understanding-global-warming-potentials</t>
+  </si>
+  <si>
+    <t>Methane Leakage Rate</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
     <t>Methane Leakage Contribution (kg CO₂e/kg H₂)</t>
   </si>
   <si>
+    <t>kg CO₂e/kg H₂</t>
+  </si>
+  <si>
     <t>Natural Gas Cost ($/GJ)</t>
   </si>
   <si>
-    <t>Frieden et al. (2024)</t>
-  </si>
-  <si>
-    <t>Key Parameters: Blue H₂ (SMR/ATR + CCS) + DAC</t>
-  </si>
-  <si>
-    <t>NATURAL GAS</t>
-  </si>
-  <si>
-    <t>$/GJ</t>
-  </si>
-  <si>
-    <t>NG Price</t>
-  </si>
-  <si>
     <t>In line with Sievert et al. (2024); NG price for 2050</t>
   </si>
   <si>
-    <t>min</t>
-  </si>
-  <si>
-    <t>max</t>
-  </si>
-  <si>
-    <t>kg CO₂/kg H₂</t>
-  </si>
-  <si>
-    <t>kg CO₂e/kg H₂</t>
-  </si>
-  <si>
-    <t>Hydrogen Cost (€2022/kg H₂)</t>
-  </si>
-  <si>
-    <t>$2023/kg H₂</t>
-  </si>
-  <si>
-    <t>€2022/kg H₂</t>
+    <t>H₂ required per liter of synfuel</t>
+  </si>
+  <si>
+    <t>kg H₂/L fuel</t>
+  </si>
+  <si>
+    <t>Argonne National Lab, Modelling of the Synfuel Production Process</t>
+  </si>
+  <si>
+    <t>kg/gallon of Ft fuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 gallon = </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> liters</t>
+  </si>
+  <si>
+    <t>Range from SAF meta-analysis</t>
+  </si>
+  <si>
+    <t>CO₂ Required per Liter of Synfuel</t>
+  </si>
+  <si>
+    <t>kg CO₂/L fuel</t>
+  </si>
+  <si>
+    <t>Calculating Synfuel Emissions</t>
+  </si>
+  <si>
+    <t>Syn-Fuel emissions (SMR+CCS) CO2</t>
+  </si>
+  <si>
+    <t>gCO2eq/MJ</t>
+  </si>
+  <si>
+    <t>Syn-Fuel emissions (SMR+CCS) methane</t>
+  </si>
+  <si>
+    <t>Total Syn-Fuel emissions (SMR+CCS)</t>
+  </si>
+  <si>
+    <t>--&gt; emissions to be abated via DACCS so that we have zero synfuel emissions</t>
+  </si>
+  <si>
+    <t>Calculating DACCS needed to offset Synfuel Emissions</t>
+  </si>
+  <si>
+    <t>Total Emissions (gCO₂eq/L synfuel)</t>
+  </si>
+  <si>
+    <t>gCO₂eq/L synfuel</t>
+  </si>
+  <si>
+    <t>DACCS Requirement (kg CO₂/L synfuel)</t>
+  </si>
+  <si>
+    <t>kg CO₂/L synfuel</t>
+  </si>
+  <si>
+    <t>Calculating Synfuel Production costs</t>
+  </si>
+  <si>
+    <t>Hydrogen cost per liter of synfuel</t>
+  </si>
+  <si>
+    <t>CO2 feedstock cost per liter of synfuel</t>
+  </si>
+  <si>
+    <t>Fischer-Tropsch and refining costs</t>
+  </si>
+  <si>
+    <t>DACCS cost to offset emissions</t>
+  </si>
+  <si>
+    <t>Synfuel (SMR+CCS+DACCS) production costs)</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Median</t>
   </si>
   <si>
     <t>Syn-Fuel cost</t>
@@ -214,7 +372,7 @@
     <t>Fossil Fuel cost</t>
   </si>
   <si>
-    <t>gCO2eq/MJ</t>
+    <t>Syn-Fuel emissions (SMR+CCS+DACCS)</t>
   </si>
   <si>
     <t>Fossil Fuel emissions</t>
@@ -226,163 +384,13 @@
     <t>gCO2eq/l</t>
   </si>
   <si>
-    <t>H₂ required per liter of synfuel</t>
-  </si>
-  <si>
-    <t>kg H₂/L fuel</t>
-  </si>
-  <si>
-    <t>Min</t>
-  </si>
-  <si>
-    <t>Max</t>
-  </si>
-  <si>
-    <t>CO₂ Required per Liter of Synfuel</t>
-  </si>
-  <si>
-    <t>kg CO₂/L fuel</t>
-  </si>
-  <si>
-    <t>Calculating Synfuel Production costs</t>
-  </si>
-  <si>
-    <t>Hydrogen cost per liter of synfuel</t>
-  </si>
-  <si>
-    <t>CO2 feedstock cost per liter of synfuel</t>
-  </si>
-  <si>
-    <t>Fischer-Tropsch and refining costs</t>
-  </si>
-  <si>
-    <t>Calculating Synfuel Emissions</t>
-  </si>
-  <si>
-    <t>Hydrogen Energy Content (Lower Heating Value, LV)</t>
-  </si>
-  <si>
-    <t>1 kg H2 in LHV basis</t>
-  </si>
-  <si>
-    <t>MJ</t>
-  </si>
-  <si>
-    <t>Syn-Fuel emissions (SMR+CCS) CO2</t>
-  </si>
-  <si>
-    <t>Syn-Fuel emissions (SMR+CCS) methane</t>
-  </si>
-  <si>
-    <t>Total Syn-Fuel emissions (SMR+CCS)</t>
-  </si>
-  <si>
-    <t>NG consumption Methane</t>
-  </si>
-  <si>
-    <t>https://www.epa.gov/ghgemissions/understanding-global-warming-potentials</t>
-  </si>
-  <si>
-    <t>Methane GWP-100 potential (1 kg CH₄ = 36 kg CO₂e)</t>
-  </si>
-  <si>
-    <t>Methane Leakage Rate</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>kg CH4/kg H2</t>
-  </si>
-  <si>
-    <t>Calculating DACCS needed to offset Synfuel Emissions</t>
-  </si>
-  <si>
-    <t>Total Emissions (gCO₂eq/L synfuel)</t>
-  </si>
-  <si>
-    <t>gCO₂eq/L synfuel</t>
-  </si>
-  <si>
-    <t>DACCS Requirement (kg CO₂/L synfuel)</t>
-  </si>
-  <si>
-    <t>kg CO₂/L synfuel</t>
-  </si>
-  <si>
-    <t>DACCS cost to offset emissions</t>
-  </si>
-  <si>
-    <t>CO2 Transport</t>
-  </si>
-  <si>
-    <t>CO2 Transport Cost</t>
-  </si>
-  <si>
-    <t>Dummy value for now</t>
-  </si>
-  <si>
-    <t>CO2 Storage</t>
-  </si>
-  <si>
-    <t>CO2 Storage Cost</t>
-  </si>
-  <si>
-    <t>Synfuel (SMR+CCS+DACCS) production costs)</t>
-  </si>
-  <si>
-    <t>Syn-Fuel emissions (SMR+CCS+DACCS)</t>
-  </si>
-  <si>
-    <t>--&gt; emissions to be abated via DACCS so that we have zero synfuel emissions</t>
-  </si>
-  <si>
-    <t>Frieden et al. (2024); 2050 SMR+CCS; Fig 5</t>
-  </si>
-  <si>
-    <t>Katebah et al. (2022); 2.7: maximum carbon capture from the SMR plant using Option 1 is around 70% of the total CO2 emissions</t>
-  </si>
-  <si>
-    <t>kg/gallon of Ft fuel</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> liters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 gallon = </t>
-  </si>
-  <si>
-    <t>Argonne National Lab, Modelling of the Synfuel Production Process</t>
+    <t>Abatement cost blue hydrogen+DACCS synfuels</t>
   </si>
   <si>
     <t>Abatement cost also needed for CO2e</t>
   </si>
   <si>
     <t>Conclusion: DACCS alone remains cheaper; why would you go for blue hydrogen + DACCS then; makes no sense</t>
-  </si>
-  <si>
-    <t>Abatement cost blue hydrogen+DACCS synfuels</t>
-  </si>
-  <si>
-    <t>TO BE UPDATED WITH 25 AND 75TH RANGE OF DAC INPUT COSTS? SAME AS FOR SYNFUELS</t>
-  </si>
-  <si>
-    <t>Range from SAF meta-analysis</t>
-  </si>
-  <si>
-    <t>Median</t>
-  </si>
-  <si>
-    <t>50%</t>
-  </si>
-  <si>
-    <t>25%</t>
-  </si>
-  <si>
-    <t>75%</t>
-  </si>
-  <si>
-    <t>DACCS LCOR</t>
   </si>
 </sst>
 </file>
@@ -578,7 +586,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
@@ -650,9 +658,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -852,7 +857,9 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Sievert  Katrin" id="{21CCBCE4-09DF-4E7D-8B2E-09F3707135FE}" userId="ksievert@ethz.ch" providerId="PeoplePicker"/>
   <person displayName="Dubey  Yash" id="{BF3000E7-5871-4931-863E-623DE601BC2A}" userId="S::ydubey@ethz.ch::8ec4c660-c9fe-4bb6-9560-48a212ff7621" providerId="AD"/>
+  <person displayName="Sievert  Katrin" id="{6BE125AD-28B8-419F-97D5-01BE9A7CC081}" userId="S::ksievert@ethz.ch::bbdc6555-5085-43f3-a455-5b29f50857e1" providerId="AD"/>
 </personList>
 </file>
 
@@ -1179,18 +1186,38 @@
 </ThreadedComments>
 </file>
 
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B18" dT="2025-05-27T07:31:29.75" personId="{BF3000E7-5871-4931-863E-623DE601BC2A}" id="{61935355-D025-4334-8AB7-9AFE8C085A31}">
+    <text>@Sievert  Katrin are these emissions measured in GWP100 or GWP20? Since the multipliers are 34x and 86x, there could be quite a significant difference between these. See section 3.1 for an example: https://www.sciencedirect.com/science/article/pii/S0306261921014215?via%3Dihub#b0215</text>
+    <mentions>
+      <mention mentionpersonId="{21CCBCE4-09DF-4E7D-8B2E-09F3707135FE}" mentionId="{19C59A26-1104-444A-B100-AE67B26EA01C}" startIndex="0" length="16"/>
+    </mentions>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>841542159</xltc2:checksum>
+        <xltc2:hyperlink startIndex="198" length="84" url="https://www.sciencedirect.com/science/article/pii/S0306261921014215?via%3Dihub#b0215"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+  <threadedComment ref="B18" dT="2025-05-27T07:34:17.38" personId="{6BE125AD-28B8-419F-97D5-01BE9A7CC081}" id="{CF2AB3C0-AFC1-4E42-A10B-6B3D51C4A4A6}" parentId="{61935355-D025-4334-8AB7-9AFE8C085A31}">
+    <text>Hi Yash, I used a GWP100 multiplier (36) - I didn't use a GWP20 multiplier for methane tho, fair point!</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB317DF6-AD4E-4C2D-91E2-8E810E428F70}">
-  <dimension ref="A1:K48"/>
-  <sheetFormatPr defaultColWidth="12.33203125" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K44"/>
+  <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" style="2"/>
+    <col min="1" max="1" width="17.5703125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="2"/>
     <col min="3" max="3" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="12.33203125" style="2"/>
+    <col min="4" max="16384" width="12.28515625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1204,7 +1231,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -1212,7 +1239,7 @@
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1221,7 +1248,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1230,7 +1257,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -1239,7 +1266,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1248,7 +1275,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -1256,7 +1283,7 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
@@ -1271,7 +1298,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
@@ -1286,7 +1313,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
@@ -1294,7 +1321,7 @@
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
@@ -1309,7 +1336,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>13</v>
       </c>
@@ -1324,7 +1351,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
@@ -1336,7 +1363,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
@@ -1348,7 +1375,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>18</v>
       </c>
@@ -1360,7 +1387,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1375,7 +1402,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>22</v>
       </c>
@@ -1383,7 +1410,7 @@
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>20</v>
       </c>
@@ -1398,7 +1425,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>23</v>
       </c>
@@ -1406,7 +1433,7 @@
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -1421,7 +1448,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -1436,7 +1463,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>24</v>
       </c>
@@ -1444,7 +1471,7 @@
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -1459,7 +1486,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -1474,7 +1501,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>25</v>
       </c>
@@ -1482,7 +1509,7 @@
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>20</v>
       </c>
@@ -1497,7 +1524,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>20</v>
       </c>
@@ -1512,7 +1539,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>26</v>
       </c>
@@ -1520,7 +1547,7 @@
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
@@ -1535,7 +1562,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -1550,7 +1577,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>27</v>
       </c>
@@ -1558,7 +1585,7 @@
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>28</v>
       </c>
@@ -1573,7 +1600,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="48" t="s">
         <v>28</v>
       </c>
@@ -1581,14 +1608,13 @@
         <v>2050</v>
       </c>
       <c r="C33" s="49">
-        <f>C48-25</f>
-        <v>517.75</v>
+        <v>542</v>
       </c>
       <c r="D33" s="48" t="s">
         <v>29</v>
       </c>
       <c r="E33" s="50" t="s">
-        <v>101</v>
+        <v>30</v>
       </c>
       <c r="F33" s="50"/>
       <c r="G33" s="50"/>
@@ -1597,14 +1623,14 @@
       <c r="J33" s="50"/>
       <c r="K33" s="50"/>
     </row>
-    <row r="34" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="30" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="B35">
         <v>2024</v>
@@ -1616,12 +1642,12 @@
         <v>29</v>
       </c>
       <c r="E35" s="41" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="B36">
         <v>2050</v>
@@ -1633,17 +1659,17 @@
         <v>29</v>
       </c>
       <c r="E36" s="41" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" s="40" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="30" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="42" t="s">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="B38">
         <v>2024</v>
@@ -1655,12 +1681,12 @@
         <v>29</v>
       </c>
       <c r="E38" s="41" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" customFormat="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="42" t="s">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="B39">
         <v>2050</v>
@@ -1672,20 +1698,20 @@
         <v>29</v>
       </c>
       <c r="E39" s="41" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="21" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B40" s="22"/>
       <c r="C40" s="23"/>
       <c r="D40" s="22"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B41" s="2">
         <v>2024</v>
@@ -1694,12 +1720,12 @@
         <v>5.49</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B42" s="2">
         <v>2050</v>
@@ -1708,53 +1734,26 @@
         <v>5.6</v>
       </c>
       <c r="D42" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="21" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A43" s="21" t="s">
-        <v>66</v>
       </c>
       <c r="B43" s="22"/>
       <c r="C43" s="22"/>
       <c r="D43" s="22"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="C44" s="2">
         <v>120</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A47" s="55" t="s">
-        <v>104</v>
-      </c>
-      <c r="B47" s="55" t="s">
-        <v>105</v>
-      </c>
-      <c r="C47" s="55" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A48" s="54">
-        <v>311.69281114021061</v>
-      </c>
-      <c r="B48" s="54">
-        <v>159.66348201703261</v>
-      </c>
-      <c r="C48" s="54">
-        <v>542.75</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1764,40 +1763,40 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24B4FBF-589B-4E3C-A2F1-4BB885F501FC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24B4FBF-589B-4E3C-A2F1-4BB885F501FC}">
   <dimension ref="A1:K32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.6640625" customWidth="1"/>
-    <col min="2" max="4" width="31.6640625" customWidth="1"/>
-    <col min="5" max="5" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" customWidth="1"/>
+    <col min="1" max="1" width="47.7109375" customWidth="1"/>
+    <col min="2" max="4" width="31.7109375" customWidth="1"/>
+    <col min="5" max="5" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="36" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="36" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>46</v>
       </c>
@@ -1808,15 +1807,15 @@
         <v>2.5499999999999998</v>
       </c>
       <c r="D3" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="31" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="B4" s="32">
         <f>(B3/Inputs!$C$6)*(1+Inputs!$C$4)</f>
@@ -1827,15 +1826,15 @@
         <v>2.8899999999999997</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="B5" s="26">
         <v>1</v>
@@ -1844,16 +1843,16 @@
         <v>2.7</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>93</v>
+        <v>54</v>
       </c>
       <c r="F5" s="45"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="B6" s="27">
         <v>3.4</v>
@@ -1862,15 +1861,15 @@
         <v>3.4</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="B7">
         <v>36</v>
@@ -1880,12 +1879,12 @@
       </c>
       <c r="D7" s="37"/>
       <c r="E7" s="33" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="B8" s="28">
         <v>1.6000000000000001E-3</v>
@@ -1894,15 +1893,15 @@
         <v>0.01</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="B9" s="34">
         <f>B6*B7*B8</f>
@@ -1913,13 +1912,13 @@
         <v>1.224</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="E9" s="33"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="B10" s="47">
         <f>Inputs!C42</f>
@@ -1930,15 +1929,15 @@
         <v>5.6</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="B12" s="46">
         <f>F12/I12</f>
@@ -1948,33 +1947,33 @@
         <v>0.5</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="F12">
         <v>1.38</v>
       </c>
       <c r="G12" t="s">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="H12" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="I12">
         <v>3.7854100000000002</v>
       </c>
       <c r="J12" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="K12" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="B13" s="46">
         <f>F13/I13</f>
@@ -1984,38 +1983,38 @@
         <v>3.5</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="F13">
         <v>8.56</v>
       </c>
       <c r="G13" t="s">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="I13">
         <v>3.7854100000000002</v>
       </c>
       <c r="J13" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="K13" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B17" s="32">
         <f>(B5)*1000/Inputs!$C$44</f>
@@ -2026,12 +2025,12 @@
         <v>22.5</v>
       </c>
       <c r="D17" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B18">
         <f>(B9)*1000/Inputs!$C$44</f>
@@ -2042,12 +2041,12 @@
         <v>10.199999999999999</v>
       </c>
       <c r="D18" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="B19" s="24">
         <f>SUM(B17:B18)</f>
@@ -2058,29 +2057,29 @@
         <v>32.700000000000003</v>
       </c>
       <c r="D19" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="44" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B20" s="24"/>
       <c r="C20" s="24"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
     </row>
-    <row r="22" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B23" s="39">
         <f>B19*Inputs!$C$14</f>
@@ -2091,12 +2090,12 @@
         <v>1134.3499200000003</v>
       </c>
       <c r="D23" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B24" s="20">
         <f>B23/1000</f>
@@ -2107,27 +2106,27 @@
         <v>1.1343499200000002</v>
       </c>
       <c r="D24" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="17"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="17"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
     </row>
-    <row r="27" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" s="35" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="B28" s="12">
         <f>'Study Parameters'!B3*'Study Parameters'!B12</f>
@@ -2141,25 +2140,25 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="B29" s="12">
         <f>(Inputs!$C$33/1000)*B13</f>
-        <v>1.1707952375039956</v>
+        <v>1.225632097976177</v>
       </c>
       <c r="C29" s="12">
         <f>(Inputs!$C$33/1000)*C13</f>
-        <v>1.8121250000000002</v>
+        <v>1.8970000000000002</v>
       </c>
       <c r="D29" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:11" s="52" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" s="52" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="52" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="B30" s="52">
         <v>0.3</v>
@@ -2172,37 +2171,37 @@
       </c>
       <c r="E30" s="53"/>
       <c r="K30" s="52" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B31" s="12">
         <f>B24*((Inputs!$C$33+Inputs!$C$36+Inputs!$C$39)/1000)</f>
-        <v>0.18762510761280002</v>
+        <v>0.19600817322240002</v>
       </c>
       <c r="C31" s="12">
         <f>C24*((Inputs!$C$33+Inputs!$C$36+Inputs!$C$39)/1000)</f>
-        <v>0.61566841908000003</v>
+        <v>0.64317640464000003</v>
       </c>
       <c r="D31" t="s">
         <v>21</v>
       </c>
       <c r="E31" s="19"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B32" s="20">
         <f>SUM(B28:B31)</f>
-        <v>2.2781682720256375</v>
+        <v>2.3413881981074187</v>
       </c>
       <c r="C32" s="20">
         <f>SUM(C28:C31)</f>
-        <v>5.2027934190800007</v>
+        <v>5.3151764046400007</v>
       </c>
       <c r="D32" s="17" t="s">
         <v>21</v>
@@ -2220,30 +2219,31 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
+  <legacyDrawing r:id="rId9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15B90E37-756A-4C57-9113-106741692D73}">
   <dimension ref="B2:F17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="97.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B2" s="56">
+    <row r="2" spans="2:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B2" s="55">
         <v>2050</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
       <c r="F2" s="40"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="14" t="s">
         <v>0</v>
       </c>
@@ -2251,35 +2251,35 @@
         <v>3</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>57</v>
+        <v>92</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="14" t="s">
-        <v>49</v>
+        <v>95</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="16">
         <f>'Study Parameters'!B32</f>
-        <v>2.2781682720256375</v>
+        <v>2.3413881981074187</v>
       </c>
       <c r="E4" s="16">
         <f>'Study Parameters'!C32</f>
-        <v>5.2027934190800007</v>
+        <v>5.3151764046400007</v>
       </c>
       <c r="F4" s="15"/>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
-        <v>50</v>
+        <v>96</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>21</v>
@@ -2294,12 +2294,12 @@
       </c>
       <c r="F5" s="15"/>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="14" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="D6" s="16">
         <v>0</v>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="F6" s="15"/>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="14" t="s">
-        <v>52</v>
+        <v>98</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="D7" s="16">
         <f>Inputs!C12</f>
@@ -2326,12 +2326,12 @@
       </c>
       <c r="F7" s="15"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="14" t="s">
-        <v>53</v>
+        <v>99</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="D8" s="16">
         <f>D7-D6</f>
@@ -2343,12 +2343,12 @@
       </c>
       <c r="F8" s="15"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="14" t="s">
-        <v>53</v>
+        <v>99</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>54</v>
+        <v>100</v>
       </c>
       <c r="D9" s="25">
         <f>D8*Inputs!$C$14</f>
@@ -2360,37 +2360,37 @@
       </c>
       <c r="F9" s="15"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="43">
         <f>(D4-D5) / D9 * 10^6</f>
-        <v>480.39774954323769</v>
+        <v>500.9439287508041</v>
       </c>
       <c r="E10" s="43">
         <f>(E4-E5) / E9 * 10^6</f>
-        <v>1430.8871934663775</v>
+        <v>1467.4111362215485</v>
       </c>
       <c r="F10" s="43">
         <f>MEDIAN(D10:E10)</f>
-        <v>955.64247150480765</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+        <v>984.17753248617623</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="51" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="51" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" s="54"/>
     </row>
   </sheetData>
@@ -2398,6 +2398,5 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>